<commit_message>
Act.0.20: Actualizo el excel BD
</commit_message>
<xml_diff>
--- a/docs/AHI_Kappa_Relaciones_Definiciones_BD.xlsx
+++ b/docs/AHI_Kappa_Relaciones_Definiciones_BD.xlsx
@@ -1047,199 +1047,199 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1496,1169 +1496,1169 @@
   <dimension ref="A1:F79"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="53.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="3.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="3.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="53.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>2023</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="8" t="s">
+      <c r="B8" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="B10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="B11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="8" t="s">
+      <c r="B12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="9" t="s">
+      <c r="B17" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="9" t="s">
+      <c r="B18" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="9" t="s">
+      <c r="B19" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="B20" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="10" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="9" t="s">
+      <c r="B21" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="9" t="s">
+      <c r="B22" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="10" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="12" t="n">
         <v>2023</v>
       </c>
-      <c r="E25" s="12"/>
+      <c r="E25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="12" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="14" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" s="15" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="16" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C31" s="16" t="s">
+      <c r="B31" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="16" t="n">
+      <c r="D31" s="17" t="n">
         <v>1544943820224710</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="B32" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" s="16" t="s">
+      <c r="B32" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C32" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="16" t="n">
+      <c r="D32" s="17" t="n">
         <v>14606741573033700</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="17" t="s">
+      <c r="D33" s="18" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="17" t="s">
+      <c r="D34" s="18" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="17" t="s">
+      <c r="C35" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D35" s="17" t="s">
+      <c r="D35" s="18" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B36" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="D36" s="17" t="s">
+      <c r="D36" s="18" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C37" s="17" t="s">
+      <c r="B37" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="18" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C38" s="17" t="s">
+      <c r="B38" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="18" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B39" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C39" s="17" t="s">
+      <c r="B39" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="18" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B40" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C40" s="17" t="s">
+      <c r="B40" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="18" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C41" s="17" t="s">
+      <c r="B41" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C41" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="18" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C42" s="17" t="s">
+      <c r="B42" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="18" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D44" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="18" t="s">
+      <c r="A45" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B45" s="18" t="s">
+      <c r="B45" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C45" s="18" t="s">
+      <c r="C45" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="D45" s="18" t="s">
+      <c r="D45" s="19" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="19" t="s">
+      <c r="A46" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="B46" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D46" s="20" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="19" t="s">
+      <c r="C47" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D47" s="20" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
+      <c r="A48" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C48" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D48" s="15" t="s">
+      <c r="D48" s="16" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="20" t="s">
+      <c r="A49" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="B49" s="20" t="s">
+      <c r="B49" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="C49" s="20" t="s">
+      <c r="C49" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="D49" s="20" t="n">
+      <c r="D49" s="21" t="n">
         <v>45139</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="21" t="s">
+      <c r="A50" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="21" t="s">
+      <c r="B50" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C50" s="21" t="s">
+      <c r="C50" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="D50" s="21" t="n">
+      <c r="D50" s="22" t="n">
         <v>45139.6340277778</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="21" t="s">
+      <c r="A51" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B51" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="21" t="s">
+      <c r="C51" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="D51" s="21" t="n">
+      <c r="D51" s="22" t="n">
         <v>45139.6555555556</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="21" t="s">
+      <c r="A52" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="B52" s="21" t="s">
+      <c r="B52" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C52" s="21" t="s">
+      <c r="C52" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="D52" s="21" t="n">
+      <c r="D52" s="22" t="n">
         <v>45139.7173611111</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="21" t="s">
+      <c r="A53" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="21" t="s">
+      <c r="B53" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C53" s="21" t="s">
+      <c r="C53" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="D53" s="21" t="n">
+      <c r="D53" s="22" t="n">
         <v>45139.7395833333</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="22" t="s">
+      <c r="C54" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="D54" s="22" t="n">
+      <c r="D54" s="23" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="22" t="s">
+      <c r="A55" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C55" s="22" t="s">
+      <c r="C55" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="22" t="n">
+      <c r="D55" s="23" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="17" t="s">
+      <c r="A56" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C56" s="17" t="s">
+      <c r="C56" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D56" s="17" t="s">
+      <c r="D56" s="18" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
+      <c r="A57" s="11"/>
+      <c r="B57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D58" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="23" t="s">
+      <c r="A59" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="B59" s="23" t="s">
+      <c r="B59" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="23" t="s">
+      <c r="C59" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="D59" s="24" t="s">
+      <c r="D59" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="E59" s="25" t="s">
+      <c r="E59" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F59" s="26" t="s">
+      <c r="F59" s="27" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="27" t="s">
+      <c r="A60" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="B60" s="27" t="s">
+      <c r="B60" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="C60" s="27" t="s">
+      <c r="C60" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="D60" s="27" t="n">
+      <c r="D60" s="28" t="n">
         <v>45139.625</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="23" t="s">
+      <c r="A61" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="B61" s="23" t="s">
+      <c r="B61" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C61" s="23" t="s">
+      <c r="C61" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="D61" s="28" t="n">
+      <c r="D61" s="29" t="n">
         <v>223</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="23" t="s">
+      <c r="A62" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="B62" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C62" s="23" t="s">
+      <c r="B62" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C62" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="D62" s="29"/>
+      <c r="D62" s="30"/>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="23" t="s">
+      <c r="A63" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="B63" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C63" s="23" t="s">
+      <c r="B63" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C63" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="D63" s="29"/>
+      <c r="D63" s="30"/>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="23" t="s">
+      <c r="A64" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="B64" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C64" s="23" t="s">
+      <c r="B64" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="D64" s="29" t="s">
+      <c r="D64" s="30" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="30" t="s">
+      <c r="A65" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="B65" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C65" s="30" t="s">
+      <c r="B65" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C65" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="D65" s="31" t="s">
+      <c r="D65" s="32" t="s">
         <v>134</v>
       </c>
-      <c r="E65" s="25" t="s">
+      <c r="E65" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F65" s="32" t="s">
+      <c r="F65" s="33" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="30" t="s">
+      <c r="A66" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="B66" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C66" s="30" t="s">
+      <c r="B66" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C66" s="31" t="s">
         <v>137</v>
       </c>
-      <c r="D66" s="31"/>
-      <c r="E66" s="25" t="s">
+      <c r="D66" s="32"/>
+      <c r="E66" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F66" s="32" t="s">
+      <c r="F66" s="33" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="30" t="s">
+      <c r="A67" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C67" s="30" t="s">
+      <c r="B67" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C67" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="D67" s="31" t="s">
+      <c r="D67" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="E67" s="25" t="s">
+      <c r="E67" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F67" s="32" t="s">
+      <c r="F67" s="33" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="30" t="s">
+      <c r="A68" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="B68" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C68" s="30" t="s">
+      <c r="B68" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C68" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="D68" s="31" t="s">
+      <c r="D68" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="E68" s="25" t="s">
+      <c r="E68" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F68" s="32" t="s">
+      <c r="F68" s="33" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="30" t="s">
+      <c r="A69" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="B69" s="30" t="s">
+      <c r="B69" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C69" s="30" t="s">
+      <c r="C69" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="D69" s="31" t="s">
+      <c r="D69" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="E69" s="25" t="s">
+      <c r="E69" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F69" s="32" t="s">
+      <c r="F69" s="33" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="30" t="s">
+      <c r="A70" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="B70" s="30" t="s">
+      <c r="B70" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C70" s="30" t="s">
+      <c r="C70" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="D70" s="31" t="s">
+      <c r="D70" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="E70" s="25" t="s">
+      <c r="E70" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F70" s="32" t="s">
+      <c r="F70" s="33" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="31" t="s">
         <v>155</v>
       </c>
-      <c r="B71" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C71" s="30" t="s">
+      <c r="B71" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" s="31" t="s">
         <v>156</v>
       </c>
-      <c r="D71" s="31" t="s">
+      <c r="D71" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="E71" s="25" t="s">
+      <c r="E71" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F71" s="32" t="s">
+      <c r="F71" s="33" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="30" t="s">
+      <c r="A72" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="B72" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C72" s="30" t="s">
+      <c r="B72" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C72" s="31" t="s">
         <v>160</v>
       </c>
-      <c r="D72" s="33" t="s">
+      <c r="D72" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="E72" s="25" t="s">
+      <c r="E72" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F72" s="32" t="s">
+      <c r="F72" s="33" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="30" t="s">
+      <c r="A73" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="B73" s="30" t="s">
+      <c r="B73" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C73" s="30" t="s">
+      <c r="C73" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="D73" s="34" t="n">
+      <c r="D73" s="35" t="n">
         <v>9999</v>
       </c>
-      <c r="E73" s="25" t="s">
+      <c r="E73" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F73" s="32" t="s">
+      <c r="F73" s="33" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="30" t="s">
+      <c r="A74" s="31" t="s">
         <v>166</v>
       </c>
-      <c r="B74" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C74" s="30" t="s">
+      <c r="B74" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C74" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="D74" s="35" t="n">
+      <c r="D74" s="36" t="n">
         <v>45802</v>
       </c>
-      <c r="E74" s="25" t="s">
+      <c r="E74" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F74" s="32" t="s">
+      <c r="F74" s="33" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="30" t="s">
+      <c r="A75" s="31" t="s">
         <v>169</v>
       </c>
-      <c r="B75" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C75" s="30" t="s">
+      <c r="B75" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="D75" s="33" t="n">
+      <c r="D75" s="34" t="n">
         <v>45878</v>
       </c>
-      <c r="E75" s="25" t="s">
+      <c r="E75" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F75" s="32" t="s">
+      <c r="F75" s="33" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="30" t="s">
+      <c r="A76" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="B76" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C76" s="30" t="s">
+      <c r="B76" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="D76" s="34"/>
-      <c r="E76" s="25" t="s">
+      <c r="D76" s="35"/>
+      <c r="E76" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F76" s="32" t="s">
+      <c r="F76" s="33" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="30" t="s">
+      <c r="A77" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="B77" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C77" s="30" t="s">
+      <c r="B77" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C77" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="D77" s="35"/>
-      <c r="E77" s="25" t="s">
+      <c r="D77" s="36"/>
+      <c r="E77" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F77" s="32" t="s">
+      <c r="F77" s="33" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="30" t="s">
+      <c r="A78" s="31" t="s">
         <v>178</v>
       </c>
-      <c r="B78" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C78" s="30" t="s">
+      <c r="B78" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C78" s="31" t="s">
         <v>179</v>
       </c>
-      <c r="D78" s="31"/>
-      <c r="E78" s="25" t="s">
+      <c r="D78" s="32"/>
+      <c r="E78" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F78" s="32" t="s">
+      <c r="F78" s="33" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="30" t="s">
+      <c r="A79" s="31" t="s">
         <v>181</v>
       </c>
-      <c r="B79" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C79" s="30" t="s">
+      <c r="B79" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C79" s="31" t="s">
         <v>182</v>
       </c>
-      <c r="D79" s="31"/>
-      <c r="E79" s="25" t="s">
+      <c r="D79" s="32"/>
+      <c r="E79" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="F79" s="32" t="s">
+      <c r="F79" s="33" t="s">
         <v>183</v>
       </c>
     </row>
@@ -2682,69 +2682,69 @@
   <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="27.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="39" t="s">
         <v>186</v>
       </c>
-      <c r="F2" s="37"/>
+      <c r="F2" s="38"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="40" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="D3" s="42"/>
+      <c r="D3" s="33"/>
       <c r="E3" s="43" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="40" t="s">
         <v>190</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="41" t="s">
         <v>191</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="D4" s="42"/>
+      <c r="D4" s="33"/>
       <c r="E4" s="43" t="n">
         <v>3</v>
       </c>
@@ -2753,148 +2753,148 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="39" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="42" t="s">
         <v>195</v>
       </c>
-      <c r="D5" s="42"/>
+      <c r="D5" s="33"/>
       <c r="E5" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="37"/>
+      <c r="F5" s="38"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="D6" s="42"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="37"/>
+      <c r="F6" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="39" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="D7" s="42"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="43" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="37"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="42" t="s">
         <v>200</v>
       </c>
-      <c r="D8" s="42"/>
+      <c r="D8" s="33"/>
       <c r="E8" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="F8" s="37"/>
+      <c r="F8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="42" t="s">
         <v>202</v>
       </c>
-      <c r="D9" s="42"/>
+      <c r="D9" s="33"/>
       <c r="E9" s="43" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="37"/>
+      <c r="F9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="39" t="s">
         <v>203</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="41" t="s">
         <v>204</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="42" t="s">
         <v>205</v>
       </c>
-      <c r="D10" s="42"/>
+      <c r="D10" s="33"/>
       <c r="E10" s="43" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="C11" s="42" t="s">
         <v>207</v>
       </c>
-      <c r="D11" s="42"/>
+      <c r="D11" s="33"/>
       <c r="E11" s="43" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="D12" s="42"/>
+      <c r="D12" s="33"/>
       <c r="E12" s="43" t="n">
         <v>10</v>
       </c>
-      <c r="F12" s="37"/>
+      <c r="F12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="42" t="s">
         <v>211</v>
       </c>
-      <c r="D13" s="42"/>
+      <c r="D13" s="33"/>
       <c r="E13" s="43" t="n">
         <v>13</v>
       </c>
-      <c r="F13" s="37"/>
+      <c r="F13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="45" t="s">
@@ -2904,89 +2904,89 @@
       <c r="C14" s="45"/>
       <c r="D14" s="45"/>
       <c r="E14" s="45"/>
-      <c r="F14" s="37"/>
+      <c r="F14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
+      <c r="A15" s="38"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
       <c r="E15" s="46"/>
-      <c r="F15" s="37"/>
+      <c r="F15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="37" t="s">
         <v>213</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="37"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="39" t="s">
         <v>214</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="39" t="s">
         <v>215</v>
       </c>
-      <c r="F17" s="37"/>
+      <c r="F17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="47" t="s">
         <v>216</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="32" t="s">
+      <c r="B18" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="33" t="s">
         <v>217</v>
       </c>
       <c r="D18" s="43" t="s">
         <v>218</v>
       </c>
-      <c r="E18" s="42"/>
-      <c r="F18" s="37"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="47" t="s">
         <v>219</v>
       </c>
-      <c r="B19" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="32" t="s">
+      <c r="B19" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="33" t="s">
         <v>220</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>221</v>
       </c>
-      <c r="E19" s="42"/>
-      <c r="F19" s="37"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="47" t="s">
         <v>222</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="33" t="s">
         <v>223</v>
       </c>
-      <c r="C20" s="32" t="s">
+      <c r="C20" s="33" t="s">
         <v>224</v>
       </c>
       <c r="D20" s="43" t="n">
         <v>1684929490</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E20" s="33" t="s">
         <v>225</v>
       </c>
       <c r="F20" s="44" t="s">
@@ -2997,16 +2997,16 @@
       <c r="A21" s="48" t="s">
         <v>226</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="33" t="s">
         <v>227</v>
       </c>
-      <c r="C21" s="32" t="s">
+      <c r="C21" s="33" t="s">
         <v>228</v>
       </c>
       <c r="D21" s="43" t="s">
         <v>229</v>
       </c>
-      <c r="E21" s="32" t="s">
+      <c r="E21" s="33" t="s">
         <v>225</v>
       </c>
       <c r="F21" s="44" t="s">
@@ -3017,181 +3017,181 @@
       <c r="A22" s="48" t="s">
         <v>231</v>
       </c>
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="33" t="s">
         <v>233</v>
       </c>
       <c r="D22" s="43" t="n">
         <v>89</v>
       </c>
-      <c r="E22" s="32" t="s">
+      <c r="E22" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F22" s="37"/>
+      <c r="F22" s="38"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="48" t="s">
         <v>234</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="33" t="s">
         <v>235</v>
       </c>
       <c r="D23" s="43" t="n">
         <v>53</v>
       </c>
-      <c r="E23" s="32" t="s">
+      <c r="E23" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F23" s="37"/>
+      <c r="F23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="48" t="s">
         <v>236</v>
       </c>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="33" t="s">
         <v>237</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="33" t="s">
         <v>238</v>
       </c>
       <c r="D24" s="43" t="n">
         <v>10000</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="E24" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F24" s="37"/>
+      <c r="F24" s="38"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="48" t="s">
         <v>239</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="33" t="s">
         <v>240</v>
       </c>
-      <c r="C25" s="32" t="s">
+      <c r="C25" s="33" t="s">
         <v>241</v>
       </c>
       <c r="D25" s="43" t="s">
         <v>242</v>
       </c>
-      <c r="E25" s="32" t="s">
+      <c r="E25" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F25" s="37"/>
+      <c r="F25" s="38"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
         <v>243</v>
       </c>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="33" t="s">
         <v>244</v>
       </c>
-      <c r="C26" s="32" t="s">
+      <c r="C26" s="33" t="s">
         <v>245</v>
       </c>
       <c r="D26" s="43" t="n">
         <v>93</v>
       </c>
-      <c r="E26" s="32" t="s">
+      <c r="E26" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F26" s="37"/>
+      <c r="F26" s="38"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="48" t="s">
         <v>246</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="33" t="s">
         <v>240</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="33" t="s">
         <v>247</v>
       </c>
       <c r="D27" s="43" t="s">
         <v>248</v>
       </c>
-      <c r="E27" s="32" t="s">
+      <c r="E27" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F27" s="37"/>
+      <c r="F27" s="38"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
         <v>249</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="33" t="s">
         <v>250</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="33" t="s">
         <v>251</v>
       </c>
       <c r="D28" s="49" t="n">
         <v>45689</v>
       </c>
-      <c r="E28" s="32" t="s">
+      <c r="E28" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F28" s="37"/>
+      <c r="F28" s="38"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="48" t="s">
         <v>252</v>
       </c>
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="33" t="s">
         <v>250</v>
       </c>
-      <c r="C29" s="32" t="s">
+      <c r="C29" s="33" t="s">
         <v>253</v>
       </c>
       <c r="D29" s="43" t="s">
         <v>254</v>
       </c>
-      <c r="E29" s="32" t="s">
+      <c r="E29" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F29" s="37"/>
+      <c r="F29" s="38"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
         <v>255</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="33" t="s">
         <v>257</v>
       </c>
       <c r="D30" s="43" t="s">
         <v>258</v>
       </c>
-      <c r="E30" s="32" t="s">
+      <c r="E30" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F30" s="37"/>
+      <c r="F30" s="38"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="48" t="s">
         <v>259</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="33" t="s">
         <v>260</v>
       </c>
       <c r="D31" s="43" t="s">
         <v>261</v>
       </c>
-      <c r="E31" s="32" t="s">
+      <c r="E31" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="F31" s="37"/>
+      <c r="F31" s="38"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="45" t="s">
@@ -3201,15 +3201,15 @@
       <c r="C32" s="45"/>
       <c r="D32" s="45"/>
       <c r="E32" s="45"/>
-      <c r="F32" s="37"/>
+      <c r="F32" s="38"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="37"/>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
+      <c r="A33" s="38"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>